<commit_message>
dev-opencode: sort of stable functional tests
</commit_message>
<xml_diff>
--- a/tests/fixtures/expected/Test_Excell_T1.xlsx
+++ b/tests/fixtures/expected/Test_Excell_T1.xlsx
@@ -595,12 +595,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="6">
-    <numFmt numFmtId="178" formatCode="#\ ##0"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="176" formatCode="#\ ##0.00"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="#\ ##0"/>
+    <numFmt numFmtId="177" formatCode="#\ ##0.0000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="177" formatCode="#\ ##0.0000"/>
   </numFmts>
   <fonts count="24" x14ac:knownFonts="1">
     <font>

</xml_diff>